<commit_message>
Owner's calls: keep ad-libs and footfalls, drop the Unveil cue, drop the Signal/Static row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -647,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H300"/>
+  <dimension ref="A1:H299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2169,49 +2169,49 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>S037</t>
+          <t>S038</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Lore</t>
+          <t>Standing rules</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Signal / Static lore</t>
+          <t>Nothing anyone owns: no brands, currencies, crypto, borrowed art or names</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Mentioned in the shape notes; source to confirm before anything uses it</t>
+          <t>Standing rule</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Part VIII</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>S038</t>
+          <t>S039</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Nothing anyone owns: no brands, currencies, crypto, borrowed art or names</t>
+          <t>Photosensitivity: nothing flashes more than 3 times a second</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Part VIII</t>
+          <t>Part XI</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -2253,17 +2253,17 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>S039</t>
+          <t>S040</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Standing rules</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Photosensitivity: nothing flashes more than 3 times a second</t>
+          <t>Vocal ad-libs and footfalls</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Standing rule</t>
+          <t>Owner: keep</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Part XI</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
@@ -2293,14 +2293,46 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="6" t="n"/>
-      <c r="H41" s="6" t="n"/>
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>S041</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>'Unveil' cue on first placement of a block type</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Won't</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Owner: nixed; the recipe stays unused</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
@@ -4881,16 +4913,6 @@
       <c r="F299" s="6" t="n"/>
       <c r="G299" s="6" t="n"/>
       <c r="H299" s="6" t="n"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="6" t="n"/>
-      <c r="B300" s="6" t="n"/>
-      <c r="C300" s="6" t="n"/>
-      <c r="D300" s="6" t="n"/>
-      <c r="E300" s="6" t="n"/>
-      <c r="F300" s="6" t="n"/>
-      <c r="G300" s="6" t="n"/>
-      <c r="H300" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H300"/>

</xml_diff>

<commit_message>
Ctrl+F3 performance report: 30 s of frames -> perf_report.txt (percentiles, hitches, worst frames, peaks)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -890,7 +890,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Debug builds optimise hot files only</t>
+          <t>The Ctrl+F3 report tool exists (perf_report.txt); running the check awaits the owner</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -1991,12 +1991,12 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Everything is mono today</t>
+          <t>Owner: go ahead</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Claude (proposed)</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Owner expected the essence attractor to do this; today it doesn't (it only draws from convergence zones). Owner to decide whether attractors should pull The Line's pivot.</t>
+        </is>
+      </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Part XVIII</t>

</xml_diff>

<commit_message>
Stereo world sounds and footsteps on the beat
- the palette renders stereo: placed sounds (set, take, machines, music
  blocks' clave) pan toward their source and soften with distance;
  ambience spreads gently; the echo ping-pongs; pan capped at +-60 %
- Mono audio accessibility toggle
- footsteps keep the beat: crouch every other beat, walk every beat,
  sprint on 8ths; ground hardness shapes them (soft scuff and crunch,
  hard click plus a quiet knock on the chord's root/5th)
- tests: stereo placement, mono, gait timing; scope sheet updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -1991,12 +1991,12 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Owner: go ahead</t>
+          <t>Owner: go ahead. Placed sounds pan, ping-pong echo, Mono audio toggle</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2339,44 +2339,168 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="6" t="n"/>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>S042</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Footsteps on the beat, by gait and ground hardness</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Crouch/walk/sprint; soft scuffs, hard knocks in key</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="6" t="n"/>
-      <c r="H43" s="6" t="n"/>
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>S043</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Default plain as a fractal patchwork of three ground materials</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Cheap per-column noise; materials swappable</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Part II</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="6" t="n"/>
-      <c r="D44" s="6" t="n"/>
-      <c r="E44" s="6" t="n"/>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="6" t="n"/>
-      <c r="H44" s="6" t="n"/>
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>S044</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Buttons that look and feel pressable (mechanical press cue)</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Part XII</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="6" t="n"/>
-      <c r="D45" s="6" t="n"/>
-      <c r="E45" s="6" t="n"/>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="6" t="n"/>
-      <c r="H45" s="6" t="n"/>
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>S045</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Standing rules</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Privacy: no telemetry, crash reporting or hardware reading; target a modest old Windows PC</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Standing rule</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>

</xml_diff>

<commit_message>
World gen flat v2: a seeded fractal patchwork of grass, sand and pebbles on the plain
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2403,12 +2403,12 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Cheap per-column noise; materials swappable</t>
+          <t>Grass / sand / pebbles by feel underfoot; flat v2; materials swappable</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Menus: mechanical-key buttons that press in and act on release; bead-on-a-string sliders
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2445,10 +2445,14 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Keys act on release; sliders are beads on a string</t>
+        </is>
+      </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
           <t>Part XII</t>

</xml_diff>

<commit_message>
Landmark shapes: canopy cap and coil stalk (glowcap, moss canopy, fern and sprout coils)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -1171,12 +1171,12 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Deliberate, low-frequency landmarks, not scatter</t>
+          <t>Glowcap, moss canopy, fern coil, sprout coil in the library</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Scope: filtering comparison rendered, awaiting the owner's pick
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Deferred earlier for usage limits</t>
+          <t>Comparison rendered (A crisp / B bleed / C variation / D both); owner to pick one to build</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Record the owner's crafting brainstorm seeds (essence as gathered microbes, flavoured by source)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2507,14 +2507,46 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
-      <c r="D46" s="6" t="n"/>
-      <c r="E46" s="6" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
-      <c r="H46" s="6" t="n"/>
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>S046</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Crafting</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Crafting system brainstorm: gathering, representation, uses, advancement from the natural surroundings</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>After the playtest. Seed: microbes/germs gathered as essence, coloured/'flavoured' by the source's biological makeup. Owner to confirm priority.</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Part XX</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>

</xml_diff>

<commit_message>
Playtest fixes: louder footsteps, fog haze and distance filtering, no midday hitch, forgiving slide, fps cap + vsync
- footsteps +8 dB
- world shader: textures fade to anisotropic filtering with distance and
  bumps flatten (no far sparkle); aerial haze from nearby; colour bleed
  dropped (read as a halo), large-scale variation kept
- music generated a slice per frame instead of a quarter-second chunk
- shadow map redrawn into a second map a quarter of the chunks per frame,
  then swapped
- power slide: crouch and sprint in either order within 0.3-0.4 s;
  sprint 7.5 blocks/s, slide burst 10
- Graphics: frame rate limit 30-200 (default 60) and vsync toggle; the
  world sound queue follows frame time

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -1340,7 +1340,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Owner picked D (bleed + variation); built into the world shader (4.16)</t>
+          <t>Owner picked D; colour bleed dropped after the playtest (halo). Variation + distance filtering kept (4.16)</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -2549,34 +2549,130 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
-      <c r="H47" s="6" t="n"/>
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>S047</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Playtest fixes</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Footsteps louder; fog haze + distance filtering; midday hitch (music slices, sliced shadow redraw)</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>From the first playtest on the owner's rig</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>4.8, 4.16, 14.7</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>S048</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Forgiving power-slide timing; faster sprint (7.5)</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Crouch/sprint in either order within 0.3-0.4 s</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="6" t="n"/>
-      <c r="D49" s="6" t="n"/>
-      <c r="E49" s="6" t="n"/>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="6" t="n"/>
-      <c r="H49" s="6" t="n"/>
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>S049</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Rendering</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Frame rate limit 30-200 (default 60) and vsync toggle</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Graphics settings</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>12.y</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>

</xml_diff>

<commit_message>
The Line: pivot finds the spot you live in (x and z), and time runs differently near it
The pivot aimed at 32-block cell centres, so it sat up to ~20 blocks off
horizontally and took hours to move. Cells are now 16 blocks and remember
where their time was spent (mean x, z); the half-life is 30 minutes.
Save v9 stores cell positions; v7/v8 histories load at their cell centres.

Near the line the visible sky (stars, moon, clouds) races ahead of the day
clock, up to 12x on the line, and runs slow after the player leaves until
it is back in step. Sun, light and shadows keep the real clock. The star
wobble is cut to a faint 2 degrees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>The Line prototype: travelling pivot, clockwise spin</t>
+          <t>The Line prototype: travelling pivot, clockwise spin, time expression</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2078,7 +2078,11 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Playtest fixes: pivot now lands on the spot you actually spend time in x and z (16-block cells remembering where their time was spent; 30-min half-life). Expression (owner's pick): the visible sky races ahead near the line and runs slow after you leave; sun and light keep the real clock; wobble kept faint.</t>
+        </is>
+      </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
           <t>Part XVIII</t>

</xml_diff>

<commit_message>
Scope + dev pile: breaking blocks and pre-generated fracture (parked until tools are decided)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2679,24 +2679,88 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="6" t="n"/>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>S050</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Breaking blocks: how it is done, and with what tools (if any)</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Owner: comes later, once we decide what tools there are. Today a click breaks a block instantly. Priority is the owner's to set.</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Part XX</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="6" t="n"/>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="6" t="n"/>
-      <c r="H51" s="6" t="n"/>
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>S051</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Rendering</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Pre-generated fracture: a broken block splits into pieces that tumble and settle</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>Owner's idea, for with S050. Cheap by design: fracture patterns baked once per shape (a handful of variants), a few short-lived pieces per break, no per-block data. Nothing flashes.</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Part XX</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Claude (proposed)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>

</xml_diff>

<commit_message>
The first loop: a diffuser that widens The Line's band; a skippable first-steps tutorial; a starter hotbar
- pulse_diffuser takes pulse of any spin and keeps none. Its feed widens
  The Line's band: halfHeight = 1 + 2*sqrt(feed/s), up to 64, judged over
  10 s, and it narrows when unfed.
- Line intensity and time rate are measured from the band's edge, so a
  harvester above or below the line is boosted only once the band reaches it.
- A new world: harvester, pipe, chest and diffuser on slots 1-4. A
  tutorial line at a time (move, place, pipe to the chest, feed a
  diffuser, where the rest is) moves on as each is done. Enter skips it.
- F7 shows the band; diffuser textures; DESIGN 6.0 and XVIII; scope
  S061-S065 (colour-vision modes, time flux on machines).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3141,54 +3141,210 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="6" t="n"/>
-      <c r="D61" s="6" t="n"/>
-      <c r="E61" s="6" t="n"/>
-      <c r="F61" s="6" t="n"/>
-      <c r="G61" s="6" t="n"/>
-      <c r="H61" s="6" t="n"/>
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>S061</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Diffuser: spends pulse widening The Line's band (the first loop)</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>Owner's design: feed per second keeps the band wide; harvesters above/below need it</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>6.0, XVIII</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n"/>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
-      <c r="E62" s="6" t="n"/>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="n"/>
-      <c r="H62" s="6" t="n"/>
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>S062</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>First-steps tutorial on a new world, skippable</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>One line at a time, moves on as done; Enter skips</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n"/>
-      <c r="B63" s="6" t="n"/>
-      <c r="C63" s="6" t="n"/>
-      <c r="D63" s="6" t="n"/>
-      <c r="E63" s="6" t="n"/>
-      <c r="F63" s="6" t="n"/>
-      <c r="G63" s="6" t="n"/>
-      <c r="H63" s="6" t="n"/>
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>S063</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>New world starts with harvester, pipe, chest, diffuser on the hotbar</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr"/>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n"/>
-      <c r="B64" s="6" t="n"/>
-      <c r="C64" s="6" t="n"/>
-      <c r="D64" s="6" t="n"/>
-      <c r="E64" s="6" t="n"/>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="6" t="n"/>
-      <c r="H64" s="6" t="n"/>
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>S064</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Colour-vision modes, one per kind of colour blindness</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Owner: red vs blue (pulse spin) must stay unmistakable for each kind. Spin already has non-colour cues (swirl, thread hand, bead turn, corkscrew)</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>11.x</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="6" t="n"/>
-      <c r="H65" s="6" t="n"/>
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>S065</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Machines sped up or slowed by time flux</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>Owner: pipes and pulse in the air stay unaffected; harvesters are the first</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n"/>

</xml_diff>

<commit_message>
Covered grass dies back to dirt after a few game minutes (never overnight): a second scheduled-update kind
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2869,12 +2869,12 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Owner asked for a distanced look at each</t>
+          <t>docs/REVIEW_2026-09.md; perf fixes merged, proposals await the owner</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fliers: five low two-winged creatures that live one game day, aged by The Line; their deaths make grass glow or grow mold
- fliers.h/.cpp: wander low over the ground, veer from obstacles, stay near
  the player. Life runs at LineTimeRateAt, so about 2 minutes on the line.
- A death on grass leaves a vivid glowing patch that fades over 4 minutes: 8
  per-frame shader constants, slow strength changes only. On dirt or wood,
  mold_patch grows (new 'mold' texture).
- Drawn as a body plus a pair of beating wings in each flier's hue.
- F3 readout; DESIGN Part XXI; scope S056 done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2953,7 +2953,7 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Part XXI</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">

</xml_diff>

<commit_message>
A trial batch of 36 materials to sort through: land, building, industry, strange
tools/batch_textures.py builds them from about a dozen parametric recipes, so
each material is one line of parameters. All of them tile, and the seam test
covers them. Each is a plain cube block named after its texture, in the library.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -2827,12 +2827,12 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>Owner isn't thrilled with the current set; wants a large pile to choose from.</t>
+          <t>36 trial materials in the library (batch_sept.vtex), four families; waiting on the owner's sort</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Colour vision setting: five modes for the pulse colours, checked with dichromat simulations
Typical, red-weak, green-weak, blue-weak and no colour (pulse_colours.h)
recolour the beads and store icons. The test found the typical trio holds up
for dichromats, but by brightness alone blue and red nearly merge (0.09); the
no-colour mode parts them (0.59).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASriJvj4z4qcZy5Ng6MUsH
</commit_message>
<xml_diff>
--- a/docs/SCOPE_MOSCOW.xlsx
+++ b/docs/SCOPE_MOSCOW.xlsx
@@ -3285,12 +3285,12 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>Owner: red vs blue (pulse spin) must stay unmistakable for each kind. Spin already has non-colour cues (swirl, thread hand, bead turn, corkscrew)</t>
+          <t>Accessibility &gt; Colour vision: 5 modes for the pulse colours; tested with dichromat simulations (the big win: no-colour, where blue and red merged)</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">

</xml_diff>